<commit_message>
Implement Closing Price Guard and Harden Task Scheduler Pathing
- powergauge.py: Add logic to override live API prices with official OHLCV closing data for absolute precision
- autonomous_pipeline.py & daily_task.py: Apply absolute path hardening to all internal script executions to ensure reliability in Windows Task Scheduler
- state_of_the_day.xlsx: Updated with calibrated 30-day technical scores
- alpha_challenge.py: Add new gamified paper trading routine
</commit_message>
<xml_diff>
--- a/state_of_the_day.xlsx
+++ b/state_of_the_day.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Develop\StockTrading\AnalyzeFinData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C37252D-3883-4520-8359-83C24DA73088}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16960648-7939-422B-B64E-9CE55C50607E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="300" yWindow="2235" windowWidth="18945" windowHeight="18420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="450" yWindow="3000" windowWidth="18945" windowHeight="18420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Short_Long" sheetId="3" r:id="rId1"/>
@@ -2866,7 +2866,7 @@
         <v>606</v>
       </c>
       <c r="N3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P3">
         <v>0</v>
@@ -2916,7 +2916,7 @@
         <v>561</v>
       </c>
       <c r="N4" s="34">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P4">
         <v>0</v>
@@ -2965,9 +2965,8 @@
       <c r="M5" t="s">
         <v>606</v>
       </c>
-      <c r="N5"/>
-      <c r="O5">
-        <v>2</v>
+      <c r="N5">
+        <v>1</v>
       </c>
       <c r="P5">
         <v>0</v>
@@ -3016,8 +3015,7 @@
       <c r="M6" s="7" t="s">
         <v>672</v>
       </c>
-      <c r="N6"/>
-      <c r="O6">
+      <c r="N6">
         <v>1</v>
       </c>
       <c r="P6">
@@ -3069,7 +3067,7 @@
       </c>
       <c r="N7"/>
       <c r="O7">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P7">
         <v>0</v>
@@ -3118,8 +3116,8 @@
       <c r="M8" s="7" t="s">
         <v>543</v>
       </c>
-      <c r="N8">
-        <v>2</v>
+      <c r="N8" s="34">
+        <v>3</v>
       </c>
       <c r="P8">
         <v>0</v>
@@ -3168,9 +3166,8 @@
       <c r="M9" s="7" t="s">
         <v>567</v>
       </c>
-      <c r="N9"/>
-      <c r="O9">
-        <v>2</v>
+      <c r="N9">
+        <v>1</v>
       </c>
       <c r="P9">
         <v>0</v>
@@ -3219,8 +3216,7 @@
       <c r="M10" t="s">
         <v>606</v>
       </c>
-      <c r="N10"/>
-      <c r="O10">
+      <c r="N10">
         <v>1</v>
       </c>
       <c r="P10">
@@ -3268,7 +3264,7 @@
         <v>695</v>
       </c>
       <c r="N11" s="34">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P11">
         <v>0</v>
@@ -3317,8 +3313,9 @@
       <c r="M12" t="s">
         <v>384</v>
       </c>
-      <c r="N12">
-        <v>2</v>
+      <c r="N12"/>
+      <c r="O12">
+        <v>1</v>
       </c>
       <c r="P12">
         <v>0</v>
@@ -3368,7 +3365,7 @@
         <v>698</v>
       </c>
       <c r="N13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P13">
         <v>0</v>
@@ -3418,7 +3415,7 @@
         <v>543</v>
       </c>
       <c r="N14">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P14">
         <v>0</v>
@@ -3468,7 +3465,7 @@
         <v>561</v>
       </c>
       <c r="N15" s="8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P15">
         <v>1</v>
@@ -3518,7 +3515,7 @@
         <v>606</v>
       </c>
       <c r="N16" s="8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P16">
         <v>0</v>
@@ -3568,7 +3565,7 @@
         <v>561</v>
       </c>
       <c r="N17" s="8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P17">
         <v>0</v>
@@ -3617,8 +3614,8 @@
       <c r="M18" t="s">
         <v>384</v>
       </c>
-      <c r="N18" s="8">
-        <v>2</v>
+      <c r="O18">
+        <v>1</v>
       </c>
       <c r="P18">
         <v>0</v>
@@ -3667,8 +3664,8 @@
       <c r="M19" t="s">
         <v>561</v>
       </c>
-      <c r="N19" s="8">
-        <v>2</v>
+      <c r="N19" s="34">
+        <v>3</v>
       </c>
       <c r="P19">
         <v>0</v>
@@ -3717,11 +3714,11 @@
       <c r="M20" s="7" t="s">
         <v>702</v>
       </c>
-      <c r="O20">
-        <v>2</v>
+      <c r="N20" s="8">
+        <v>1</v>
       </c>
       <c r="P20">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:20">
@@ -3777,7 +3774,7 @@
         <v>598</v>
       </c>
       <c r="N27" s="34">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P27">
         <v>0</v>
@@ -3826,8 +3823,8 @@
       <c r="M28" s="7" t="s">
         <v>598</v>
       </c>
-      <c r="N28">
-        <v>2</v>
+      <c r="N28" s="34">
+        <v>3</v>
       </c>
       <c r="P28">
         <v>0</v>
@@ -3882,8 +3879,7 @@
       <c r="M29" s="49" t="s">
         <v>614</v>
       </c>
-      <c r="N29"/>
-      <c r="O29">
+      <c r="N29">
         <v>1</v>
       </c>
       <c r="P29">
@@ -3931,7 +3927,7 @@
         <v>335</v>
       </c>
       <c r="N30">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P30">
         <v>0</v>
@@ -3981,7 +3977,7 @@
         <v>543</v>
       </c>
       <c r="N31" s="34">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P31">
         <v>0</v>
@@ -4030,9 +4026,8 @@
       <c r="M32" t="s">
         <v>561</v>
       </c>
-      <c r="N32"/>
-      <c r="O32">
-        <v>2</v>
+      <c r="N32">
+        <v>1</v>
       </c>
       <c r="P32">
         <v>0</v>
@@ -4081,9 +4076,8 @@
       <c r="M33" t="s">
         <v>614</v>
       </c>
-      <c r="N33"/>
-      <c r="O33">
-        <v>2</v>
+      <c r="N33">
+        <v>1</v>
       </c>
       <c r="P33">
         <v>0</v>
@@ -4132,9 +4126,8 @@
       <c r="M34" s="7" t="s">
         <v>598</v>
       </c>
-      <c r="N34"/>
-      <c r="O34">
-        <v>4</v>
+      <c r="N34">
+        <v>1</v>
       </c>
       <c r="P34">
         <v>0</v>
@@ -4183,8 +4176,8 @@
       <c r="M35" t="s">
         <v>561</v>
       </c>
-      <c r="N35">
-        <v>2</v>
+      <c r="N35" s="34">
+        <v>3</v>
       </c>
       <c r="P35">
         <v>0</v>
@@ -4234,7 +4227,7 @@
         <v>561</v>
       </c>
       <c r="N36">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P36">
         <v>0</v>
@@ -4284,7 +4277,7 @@
         <v>561</v>
       </c>
       <c r="N37">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P37">
         <v>0</v>
@@ -4333,8 +4326,9 @@
       <c r="M38" t="s">
         <v>200</v>
       </c>
-      <c r="N38">
-        <v>2</v>
+      <c r="N38"/>
+      <c r="O38">
+        <v>1</v>
       </c>
       <c r="P38">
         <v>0</v>
@@ -4384,8 +4378,8 @@
       <c r="M39" s="7" t="s">
         <v>672</v>
       </c>
-      <c r="N39">
-        <v>2</v>
+      <c r="N39" s="34">
+        <v>3</v>
       </c>
       <c r="P39">
         <v>0</v>
@@ -4434,9 +4428,8 @@
       <c r="M40" t="s">
         <v>614</v>
       </c>
-      <c r="N40"/>
-      <c r="O40">
-        <v>2</v>
+      <c r="N40">
+        <v>1</v>
       </c>
       <c r="P40">
         <v>0</v>
@@ -4485,9 +4478,8 @@
       <c r="M41" t="s">
         <v>200</v>
       </c>
-      <c r="N41"/>
-      <c r="O41">
-        <v>2</v>
+      <c r="N41">
+        <v>1</v>
       </c>
       <c r="P41">
         <v>0</v>
@@ -4536,9 +4528,8 @@
       <c r="M42" s="7" t="s">
         <v>543</v>
       </c>
-      <c r="N42"/>
-      <c r="O42">
-        <v>2</v>
+      <c r="N42">
+        <v>1</v>
       </c>
       <c r="P42">
         <v>0</v>
@@ -4587,8 +4578,8 @@
       <c r="M43" t="s">
         <v>384</v>
       </c>
-      <c r="N43">
-        <v>2</v>
+      <c r="N43" s="34">
+        <v>3</v>
       </c>
       <c r="P43">
         <v>0</v>
@@ -4608,7 +4599,7 @@
         <v>92.51</v>
       </c>
       <c r="E44">
-        <v>98.12</v>
+        <v>105.2</v>
       </c>
       <c r="F44" s="12">
         <v>125</v>
@@ -4618,11 +4609,11 @@
       </c>
       <c r="H44" s="22">
         <f t="shared" ref="H44:H45" si="30">E44*0.92</f>
-        <v>90.270400000000009</v>
+        <v>96.784000000000006</v>
       </c>
       <c r="I44" s="9">
         <f t="shared" ref="I44:I45" si="31">F44/E44 -1</f>
-        <v>0.27395026498165498</v>
+        <v>0.18821292775665399</v>
       </c>
       <c r="J44" s="26">
         <f t="shared" ref="J44:J45" si="32">C44*D44</f>
@@ -4637,7 +4628,8 @@
       <c r="M44" s="7" t="s">
         <v>543</v>
       </c>
-      <c r="N44">
+      <c r="N44"/>
+      <c r="O44">
         <v>1</v>
       </c>
       <c r="P44">
@@ -4688,7 +4680,7 @@
         <v>561</v>
       </c>
       <c r="N45" s="34">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="P45">
         <v>0</v>
@@ -4737,8 +4729,8 @@
       <c r="M46" s="7" t="s">
         <v>543</v>
       </c>
-      <c r="N46">
-        <v>2</v>
+      <c r="N46" s="34">
+        <v>3</v>
       </c>
       <c r="P46">
         <v>0</v>
@@ -4837,8 +4829,8 @@
       <c r="M48" t="s">
         <v>614</v>
       </c>
-      <c r="N48">
-        <v>2</v>
+      <c r="N48" s="34">
+        <v>3</v>
       </c>
       <c r="P48">
         <v>0</v>
@@ -4888,7 +4880,7 @@
         <v>598</v>
       </c>
       <c r="N49" s="8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P49">
         <v>1</v>
@@ -4937,7 +4929,7 @@
       <c r="M50" t="s">
         <v>384</v>
       </c>
-      <c r="N50" s="8">
+      <c r="O50">
         <v>1</v>
       </c>
       <c r="P50">
@@ -4988,7 +4980,7 @@
         <v>543</v>
       </c>
       <c r="N51" s="8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P51">
         <v>0</v>

</xml_diff>

<commit_message>
Harden Windows UTF-8 Terminal Stream Redirection
- Implement SafeStreamWrapper in ai_portfolio_game.py, autonomous_pipeline.py, and watchdog.py
- Reconfigure sys.stdout and sys.stderr to utilize UTF-8 with replace-on-error in cp1252 consoles
- Completely prevent UnicodeEncodeError crashes when printing rich emojis headlessly in Windows Task Scheduler
</commit_message>
<xml_diff>
--- a/state_of_the_day.xlsx
+++ b/state_of_the_day.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Develop\StockTrading\AnalyzeFinData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8085171E-1F61-4790-8380-2C13092AAB5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D2BBF47-1491-4C8A-8567-74CBF6AA4163}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="660" yWindow="1605" windowWidth="18825" windowHeight="18420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4111" uniqueCount="720">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4114" uniqueCount="720">
   <si>
     <t>Symb</t>
   </si>
@@ -2894,7 +2894,8 @@
       <c r="M3" s="49" t="s">
         <v>606</v>
       </c>
-      <c r="N3">
+      <c r="N3"/>
+      <c r="O3">
         <v>1</v>
       </c>
       <c r="P3">
@@ -2945,7 +2946,7 @@
         <v>561</v>
       </c>
       <c r="N4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P4">
         <v>0</v>
@@ -2994,8 +2995,7 @@
       <c r="M5" t="s">
         <v>606</v>
       </c>
-      <c r="N5"/>
-      <c r="O5">
+      <c r="N5">
         <v>1</v>
       </c>
       <c r="P5">
@@ -3046,7 +3046,7 @@
         <v>672</v>
       </c>
       <c r="N6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P6">
         <v>0</v>
@@ -3095,8 +3095,8 @@
       <c r="M7" t="s">
         <v>384</v>
       </c>
-      <c r="N7">
-        <v>2</v>
+      <c r="N7" s="34">
+        <v>3</v>
       </c>
       <c r="P7">
         <v>0</v>
@@ -3197,7 +3197,7 @@
       </c>
       <c r="N9"/>
       <c r="O9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P9">
         <v>0</v>
@@ -3246,9 +3246,8 @@
       <c r="M10" t="s">
         <v>606</v>
       </c>
-      <c r="N10"/>
-      <c r="O10">
-        <v>2</v>
+      <c r="N10">
+        <v>1</v>
       </c>
       <c r="P10">
         <v>0</v>
@@ -3295,7 +3294,7 @@
         <v>695</v>
       </c>
       <c r="N11" s="34">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="P11">
         <v>0</v>
@@ -3346,7 +3345,7 @@
       </c>
       <c r="N12"/>
       <c r="O12">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P12">
         <v>0</v>
@@ -3397,7 +3396,7 @@
       </c>
       <c r="N13"/>
       <c r="O13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P13">
         <v>0</v>
@@ -3448,10 +3447,10 @@
       </c>
       <c r="N14"/>
       <c r="O14">
+        <v>2</v>
+      </c>
+      <c r="P14">
         <v>1</v>
-      </c>
-      <c r="P14">
-        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:18">
@@ -3498,7 +3497,7 @@
         <v>561</v>
       </c>
       <c r="N15">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P15">
         <v>0</v>
@@ -3547,7 +3546,7 @@
       <c r="M16" t="s">
         <v>384</v>
       </c>
-      <c r="N16" s="8">
+      <c r="O16">
         <v>1</v>
       </c>
       <c r="P16">
@@ -3568,7 +3567,7 @@
         <v>14.18</v>
       </c>
       <c r="E17">
-        <v>14.23</v>
+        <v>14.63</v>
       </c>
       <c r="F17" s="12">
         <v>17.5</v>
@@ -3577,15 +3576,15 @@
         <v>13</v>
       </c>
       <c r="H17" s="22">
-        <f t="shared" ref="H17:H19" si="12">E17*0.92</f>
-        <v>13.091600000000001</v>
+        <f t="shared" ref="H17:H20" si="12">E17*0.92</f>
+        <v>13.459600000000002</v>
       </c>
       <c r="I17" s="9">
-        <f t="shared" ref="I17:I19" si="13">F17/E17 -1</f>
-        <v>0.2297962052002811</v>
+        <f t="shared" ref="I17:I20" si="13">F17/E17 -1</f>
+        <v>0.19617224880382778</v>
       </c>
       <c r="J17" s="26">
-        <f t="shared" ref="J17:J19" si="14">C17*D17</f>
+        <f t="shared" ref="J17:J20" si="14">C17*D17</f>
         <v>1843.3999999999999</v>
       </c>
       <c r="K17" s="18">
@@ -3599,7 +3598,7 @@
       </c>
       <c r="N17"/>
       <c r="O17">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P17">
         <v>1</v>
@@ -3648,12 +3647,11 @@
       <c r="M18" s="7" t="s">
         <v>702</v>
       </c>
-      <c r="N18"/>
-      <c r="O18">
+      <c r="N18">
         <v>1</v>
       </c>
       <c r="P18">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:20">
@@ -3699,7 +3697,7 @@
       <c r="M19" s="7" t="s">
         <v>567</v>
       </c>
-      <c r="O19">
+      <c r="N19" s="8">
         <v>1</v>
       </c>
       <c r="P19">
@@ -3710,6 +3708,51 @@
       <c r="A20">
         <v>18</v>
       </c>
+      <c r="B20" t="s">
+        <v>705</v>
+      </c>
+      <c r="C20" s="5">
+        <v>95</v>
+      </c>
+      <c r="D20">
+        <v>11.55</v>
+      </c>
+      <c r="E20">
+        <v>11.55</v>
+      </c>
+      <c r="F20" s="12">
+        <v>25</v>
+      </c>
+      <c r="G20" s="26">
+        <v>10</v>
+      </c>
+      <c r="H20" s="22">
+        <f t="shared" si="12"/>
+        <v>10.626000000000001</v>
+      </c>
+      <c r="I20" s="9">
+        <f t="shared" si="13"/>
+        <v>1.1645021645021645</v>
+      </c>
+      <c r="J20" s="26">
+        <f t="shared" si="14"/>
+        <v>1097.25</v>
+      </c>
+      <c r="K20" s="18">
+        <v>46197</v>
+      </c>
+      <c r="L20" t="s">
+        <v>276</v>
+      </c>
+      <c r="M20" t="s">
+        <v>200</v>
+      </c>
+      <c r="N20" s="8">
+        <v>1</v>
+      </c>
+      <c r="P20">
+        <v>0</v>
+      </c>
     </row>
     <row r="24" spans="1:20">
       <c r="T24" s="7"/>
@@ -3763,7 +3806,8 @@
       <c r="M27" s="7" t="s">
         <v>598</v>
       </c>
-      <c r="N27">
+      <c r="N27"/>
+      <c r="O27">
         <v>1</v>
       </c>
       <c r="P27">
@@ -3814,7 +3858,7 @@
         <v>598</v>
       </c>
       <c r="N28" s="34">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P28">
         <v>0</v>
@@ -3870,7 +3914,7 @@
         <v>614</v>
       </c>
       <c r="N29">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P29">
         <v>0</v>
@@ -3917,7 +3961,7 @@
         <v>335</v>
       </c>
       <c r="N30">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P30">
         <v>0</v>
@@ -3968,7 +4012,7 @@
       </c>
       <c r="N31"/>
       <c r="O31">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P31">
         <v>0</v>
@@ -4017,8 +4061,9 @@
       <c r="M32" t="s">
         <v>561</v>
       </c>
-      <c r="N32" s="34">
-        <v>3</v>
+      <c r="N32"/>
+      <c r="O32">
+        <v>1</v>
       </c>
       <c r="P32">
         <v>0</v>
@@ -4067,8 +4112,7 @@
       <c r="M33" t="s">
         <v>614</v>
       </c>
-      <c r="N33"/>
-      <c r="O33">
+      <c r="N33">
         <v>1</v>
       </c>
       <c r="P33">
@@ -4118,8 +4162,9 @@
       <c r="M34" s="7" t="s">
         <v>598</v>
       </c>
-      <c r="N34" s="34">
-        <v>3</v>
+      <c r="N34"/>
+      <c r="O34">
+        <v>1</v>
       </c>
       <c r="P34">
         <v>0</v>
@@ -4170,7 +4215,7 @@
       </c>
       <c r="N35"/>
       <c r="O35">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P35">
         <v>0</v>
@@ -4220,7 +4265,7 @@
         <v>561</v>
       </c>
       <c r="N36" s="34">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P36">
         <v>0</v>
@@ -4269,8 +4314,7 @@
       <c r="M37" t="s">
         <v>561</v>
       </c>
-      <c r="N37"/>
-      <c r="O37">
+      <c r="N37">
         <v>1</v>
       </c>
       <c r="P37">
@@ -4320,8 +4364,8 @@
       <c r="M38" t="s">
         <v>200</v>
       </c>
-      <c r="N38">
-        <v>2</v>
+      <c r="N38" s="34">
+        <v>3</v>
       </c>
       <c r="P38">
         <v>0</v>
@@ -4371,9 +4415,8 @@
       <c r="M39" s="7" t="s">
         <v>672</v>
       </c>
-      <c r="N39"/>
-      <c r="O39">
-        <v>2</v>
+      <c r="N39">
+        <v>1</v>
       </c>
       <c r="P39">
         <v>0</v>
@@ -4423,7 +4466,7 @@
         <v>614</v>
       </c>
       <c r="N40" s="34">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P40">
         <v>0</v>
@@ -4473,7 +4516,7 @@
         <v>200</v>
       </c>
       <c r="N41" s="34">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P41">
         <v>0</v>
@@ -4524,7 +4567,7 @@
       </c>
       <c r="N42"/>
       <c r="O42">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P42">
         <v>0</v>
@@ -4573,9 +4616,8 @@
       <c r="M43" t="s">
         <v>384</v>
       </c>
-      <c r="N43"/>
-      <c r="O43">
-        <v>2</v>
+      <c r="N43">
+        <v>1</v>
       </c>
       <c r="P43">
         <v>0</v>
@@ -4624,8 +4666,8 @@
       <c r="M44" s="7" t="s">
         <v>543</v>
       </c>
-      <c r="N44">
-        <v>2</v>
+      <c r="N44" s="34">
+        <v>3</v>
       </c>
       <c r="P44">
         <v>1</v>
@@ -4674,8 +4716,7 @@
       <c r="M45" t="s">
         <v>561</v>
       </c>
-      <c r="N45"/>
-      <c r="O45">
+      <c r="N45">
         <v>1</v>
       </c>
       <c r="P45">
@@ -4727,7 +4768,7 @@
       </c>
       <c r="N46"/>
       <c r="O46">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P46">
         <v>0</v>
@@ -4777,7 +4818,7 @@
         <v>543</v>
       </c>
       <c r="O47">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P47">
         <v>0</v>
@@ -4797,7 +4838,7 @@
         <v>57.3</v>
       </c>
       <c r="E48">
-        <v>57.43</v>
+        <v>57.81</v>
       </c>
       <c r="F48" s="12">
         <v>62</v>
@@ -4807,11 +4848,11 @@
       </c>
       <c r="H48" s="22">
         <f t="shared" si="36"/>
-        <v>52.835599999999999</v>
+        <v>53.185200000000002</v>
       </c>
       <c r="I48" s="9">
         <f t="shared" si="37"/>
-        <v>7.9575134946891835E-2</v>
+        <v>7.2478809894481966E-2</v>
       </c>
       <c r="J48" s="26">
         <f t="shared" si="38"/>
@@ -4828,7 +4869,7 @@
       </c>
       <c r="N48"/>
       <c r="O48">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P48">
         <v>1</v>
@@ -4878,7 +4919,7 @@
         <v>598</v>
       </c>
       <c r="N49">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P49">
         <v>0</v>
@@ -4928,7 +4969,7 @@
         <v>543</v>
       </c>
       <c r="N50" s="34">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P50">
         <v>0</v>
@@ -14003,7 +14044,7 @@
     </row>
     <row r="179" spans="2:20">
       <c r="B179" s="14">
-        <v>4</v>
+        <v>-5</v>
       </c>
       <c r="C179" s="14"/>
       <c r="D179" t="s">

</xml_diff>